<commit_message>
benchmarks(joints): rj008's column set is bounded by the back joint
The rj008 builder clipped its column region to the section's right edge at
x = 72.407 rather than to the back joint at x = 68.4, so the set came out as
thirteen chains, three of them running on past the back joint into the strip the
vendor leaves uncut and carrying 24 m of trace the vendor's model has no
counterpart for.

Bounded by the two joints the vendor bounds it by, the set is the vendor's own:
twelve chains, the three highest ending ON the back joint at y = 6.032, 16.192
and 26.352, 301.555 m of column trace and 389.462 m of joint in all.

The factor does not move. FS 0.764 on a bracket of [0.75390625, 0.7734375],
nine of nine trials decided, longest 1,221 sweeps. verify_rebuild.py --group
joints reproduces all 23 targets with only rj008.xlsx changed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj008.xlsx
+++ b/docs/verification/files/rocscience/joints/rj008.xlsx
@@ -5378,10 +5378,10 @@
         <v>36.5</v>
       </c>
       <c r="E15" s="3">
-        <v>68.4185768851</v>
+        <v>68.4</v>
       </c>
       <c r="F15" s="3">
-        <v>6.0</v>
+        <v>6.0321761089</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3">
@@ -5415,10 +5415,10 @@
         <v>36.5</v>
       </c>
       <c r="E16" s="3">
-        <v>72.407</v>
+        <v>68.4</v>
       </c>
       <c r="F16" s="3">
-        <v>9.2518485229</v>
+        <v>16.1921761089</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3">
@@ -5452,10 +5452,10 @@
         <v>36.5</v>
       </c>
       <c r="E17" s="3">
-        <v>72.407</v>
+        <v>68.4</v>
       </c>
       <c r="F17" s="3">
-        <v>19.4118485229</v>
+        <v>26.3521761089</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3">
@@ -5477,37 +5477,19 @@
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>col-13</t>
-        </is>
-      </c>
-      <c r="C18" s="3">
-        <v>68.4070298797</v>
-      </c>
-      <c r="D18" s="3">
-        <v>36.5</v>
-      </c>
-      <c r="E18" s="3">
-        <v>72.407</v>
-      </c>
-      <c r="F18" s="3">
-        <v>29.5718485229</v>
-      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="3"/>
-      <c r="H18" s="3">
-        <v>39.0</v>
-      </c>
+      <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
-      <c r="M18" s="3">
-        <v>15000000.0</v>
-      </c>
-      <c r="N18" s="3">
-        <v>10000000.0</v>
-      </c>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
       <c r="O18" s="3"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>